<commit_message>
architecture and test addition in GP
</commit_message>
<xml_diff>
--- a/tests/data/gravure_printing_test.xlsx
+++ b/tests/data/gravure_printing_test.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="74">
   <si>
     <t xml:space="preserve">Experiment Info</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">Variation</t>
   </si>
   <si>
+    <t xml:space="preserve">Architecture</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sample dimension</t>
   </si>
   <si>
@@ -188,6 +191,9 @@
   </si>
   <si>
     <t xml:space="preserve">1000 rpm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nip</t>
   </si>
   <si>
     <t xml:space="preserve">1 cm x 1 cm</t>
@@ -612,7 +618,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AY3"/>
+  <dimension ref="A1:AZ3"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17"/>
@@ -622,46 +628,46 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="26" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="36" style="1" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="47" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="1" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="1" width="41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="37" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="48" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="1" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="1" width="41"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -685,10 +691,10 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2"/>
+      <c r="T1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="T1" s="3"/>
       <c r="U1" s="3"/>
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
@@ -720,6 +726,7 @@
       <c r="AW1" s="3"/>
       <c r="AX1" s="3"/>
       <c r="AY1" s="3"/>
+      <c r="AZ1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
@@ -776,7 +783,7 @@
       <c r="R2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" s="4" t="s">
         <v>20</v>
       </c>
       <c r="T2" s="5" t="s">
@@ -792,10 +799,10 @@
         <v>24</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="Z2" s="5" t="s">
         <v>26</v>
@@ -874,168 +881,174 @@
       </c>
       <c r="AY2" s="5" t="s">
         <v>51</v>
+      </c>
+      <c r="AZ2" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F3" s="1" t="str">
         <f aca="false">CONCATENATE("SAU_",B3,"_",C3,"_",D3,"_C-",E3)</f>
         <v>SAU_GeSo_1_1_C-1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I3" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J3" s="1" t="n">
         <v>0.16</v>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="K3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="L3" s="1" t="n">
         <v>0.16</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="M3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="N3" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="O3" s="1" t="n">
         <v>90</v>
       </c>
-      <c r="O3" s="1" t="n">
+      <c r="P3" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="P3" s="1" t="n">
+      <c r="Q3" s="1" t="n">
         <v>150</v>
       </c>
-      <c r="Q3" s="1" t="n">
+      <c r="R3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="R3" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="S3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA3" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AC3" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="AD3" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="AE3" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG3" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH3" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AJ3" s="1" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AL3" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AM3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN3" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AP3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="AQ3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AR3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AS3" s="1" t="n">
+        <v>120</v>
+      </c>
+      <c r="AT3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="AU3" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="AV3" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AW3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="AY3" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="T3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="U3" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="W3" s="1" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z3" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AA3" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="AB3" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="AC3" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="AD3" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="AF3" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG3" s="1" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI3" s="1" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK3" s="1" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AL3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM3" s="1" t="n">
-        <v>150</v>
-      </c>
-      <c r="AN3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AO3" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="AP3" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AQ3" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="AR3" s="1" t="n">
-        <v>120</v>
-      </c>
-      <c r="AS3" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="AT3" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="AU3" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AV3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="AW3" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="AX3" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="AY3" s="1" t="n">
+      <c r="AZ3" s="1" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="S1:AY1"/>
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="T1:AZ1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>